<commit_message>
Add initial configuration and schematic files for STM32 project
- Created OpenOCD configuration file for STM32 development.
- Added schematic text file containing detailed circuit design.
- Included binary files for original release image and STM32 flash.
- Added schematic images for better visualization of the design.
</commit_message>
<xml_diff>
--- a/Hardware Design/BOM_UMH 7_UMH 7_2026-09-02.xlsx
+++ b/Hardware Design/BOM_UMH 7_UMH 7_2026-09-02.xlsx
@@ -20,7 +20,7 @@
     <t xml:space="preserve">Bill of Materials </t>
   </si>
   <si>
-    <t>BOM_UMH 7_UMH 7_2026-09-02</t>
+    <t>BOM_UMH 7_UMH 7_2026-09-08</t>
   </si>
   <si>
     <t>Project Title：</t>
@@ -38,7 +38,7 @@
     <t>Report Time：</t>
   </si>
   <si>
-    <t>2026年9月2日 14:39:54</t>
+    <t>2026年9月8日 13:11:35</t>
   </si>
   <si>
     <t>No.</t>
@@ -845,13 +845,13 @@
     <t>Report Time</t>
   </si>
   <si>
-    <t>14:39:54</t>
+    <t>13:11:35</t>
   </si>
   <si>
     <t>Report Date</t>
   </si>
   <si>
-    <t>2026年9月2日</t>
+    <t>2026年9月8日</t>
   </si>
   <si>
     <t>Report Date&amp;Time</t>

</xml_diff>